<commit_message>
Add the missed MOR findings and require a second pass plus prompt updates.
The review skill now says to reread the file after the checklist, append anything
the checklist missed to the same workbook, and fold new checks into GROK-PROMPT
whenever a revised final is compared.

Co-authored-by: peterli0913 <peterli0913@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/L2-Step1-MOR-硬伤清单_10-28-2026.xlsx
+++ b/L2-Step1-MOR-硬伤清单_10-28-2026.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MOR 硬伤" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'MOR 硬伤'!$A$1:$F$57</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'MOR 硬伤'!$A$1:$F$61</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -458,7 +458,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:F57"/>
+  <dimension ref="A1:F61"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -1007,7 +1007,7 @@
       </c>
       <c r="F18" s="2" t="inlineStr">
         <is>
-          <t>★上下限仍是占位符 “X oC”。按 3.20 等应为 15–25 °C。</t>
+          <t>★上下限仍是占位符 “X oC”，应按 15–25 °C。紧接着的超温预警是 22–28 °C，本步控温却是 20±5 °C：目标 20 °C 已经低于预警低限，正常加料会一直报警，高限 28 °C 又高于 NOR 上限 25 °C。3.20.7、3.23.7、3.26.7 等同类 DIC 步的预警是 17–23 °C。这里改为 17–23 °C。</t>
         </is>
       </c>
     </row>
@@ -1127,7 +1127,7 @@
       </c>
       <c r="F22" s="2" t="inlineStr">
         <is>
-          <t>预警写成 低限 22 °C、高限 23 °C，低限比目标 20 °C 还高，加料过程会一直报警。其他氨基酸为 17–23 °C。改为 17–23 °C。</t>
+          <t>预警写成 低限 22 °C、高限 23 °C，低限比目标 20 °C 还高，加料过程会一直报警。3.20.7 等同类步骤为 17–23 °C（3.17.7 是另一套 22–28 °C，见该行）。改为 17–23 °C。</t>
         </is>
       </c>
     </row>
@@ -1507,17 +1507,17 @@
       </c>
       <c r="D35" s="3" t="inlineStr">
         <is>
-          <t>3.28（Leu16 前脱保护）第二次再溶胀</t>
+          <t>3.7.6 Phe23；3.10.5、3.18.5 的不合格处置</t>
         </is>
       </c>
       <c r="E35" s="3" t="inlineStr">
         <is>
-          <t>3.25.8 DMF addition</t>
+          <t>NMT 841 min</t>
         </is>
       </c>
       <c r="F35" s="3" t="inlineStr">
         <is>
-          <t>3.28 节里这一步编号写成 3.25.8，应为 3.28.8（全文两处，3.28 节那处错）。</t>
+          <t>Phe23 的偶联上限中英文都写 841 min，其余氨基酸写 840 min。3.10.5（NMeAsn22）、3.18.5（Ser20）本步上限是 840 min，不合格后继续取样的处置句仍写 841 min，处置比本步上限多 1 min。Phe23 改为 840 min；两处处置句改成与本步上限相同。</t>
         </is>
       </c>
     </row>
@@ -1537,17 +1537,17 @@
       </c>
       <c r="D36" s="2" t="inlineStr">
         <is>
-          <t>3.13 Asn21；3.43；3.2.5</t>
+          <t>3.22.8 与 3.22.9</t>
         </is>
       </c>
       <c r="E36" s="2" t="inlineStr">
         <is>
-          <t>documented in Ins3.43.2</t>
+          <t>3.22.9 Resin reswelling wash 2</t>
         </is>
       </c>
       <c r="F36" s="2" t="inlineStr">
         <is>
-          <t>交叉引用中英不一致：3.13 英文 “Ins3.13.5”、中文“3.13.7”；3.43 一处英文 3.43.2、中文 3.42.2；3.2.5 一处英文 3.1.3、中文 3.2.1。核对后统一。</t>
+          <t>3.22.8 已经是“溶胀后洗涤2”（加 12 V DMF）。3.22.9 不再加液，只鼓氮气、搅拌、排液，标题仍写洗涤2。批记录里同一次洗涤会出现两个“洗涤2”。3.22.9 改成该步的排液记录，或并入 3.22.8。</t>
         </is>
       </c>
     </row>
@@ -1567,17 +1567,17 @@
       </c>
       <c r="D37" s="3" t="inlineStr">
         <is>
-          <t>版本说明 第 3 条</t>
+          <t>3.44 树脂洗涤</t>
         </is>
       </c>
       <c r="E37" s="3" t="inlineStr">
         <is>
-          <t>20±10 min (target: 10 min)</t>
+          <t>3.44.1 Sample</t>
         </is>
       </c>
       <c r="F37" s="3" t="inlineStr">
         <is>
-          <t>版本说明写封端 DIPEA 参考加料时间目标 10 min，3.4.3 正文写 20 ± 10 min（目标 20 min）。</t>
+          <t>3.44.1 用了两次：前面是脱保护后 IPAc 洗涤，这里是第 2 次洗涤的氯冉酸取样。两个操作不能共用一个指令号。取样改为 3.44.2。（3.43.5 同样把洗涤和 IPC 编成同一个号。）</t>
         </is>
       </c>
     </row>
@@ -1597,17 +1597,17 @@
       </c>
       <c r="D38" s="2" t="inlineStr">
         <is>
-          <t>3.17.8、3.26.8 活化</t>
+          <t>3.28（Leu16 前脱保护）第二次再溶胀</t>
         </is>
       </c>
       <c r="E38" s="2" t="inlineStr">
         <is>
-          <t>Maintain for NLT 15 min</t>
+          <t>3.25.8 DMF addition</t>
         </is>
       </c>
       <c r="F38" s="2" t="inlineStr">
         <is>
-          <t>英文 NLT 15 min（目标 20 min），中文 20 ± 5 min；参数表 NOR 15–25 min。中文优先，英文改为 20 ± 5 min。</t>
+          <t>3.28 节里这一步编号写成 3.25.8，应为 3.28.8（全文两处，3.28 节那处错）。</t>
         </is>
       </c>
     </row>
@@ -1627,17 +1627,17 @@
       </c>
       <c r="D39" s="3" t="inlineStr">
         <is>
-          <t>3.0 预处理</t>
+          <t>3.13 Asn21；3.43；3.2.5</t>
         </is>
       </c>
       <c r="E39" s="3" t="inlineStr">
         <is>
-          <t>搅拌5 min±5 min</t>
+          <t>documented in Ins3.43.2</t>
         </is>
       </c>
       <c r="F39" s="3" t="inlineStr">
         <is>
-          <t>英文 5 ± 2 min，中文 5 ± 5 min。</t>
+          <t>交叉引用中英不一致：3.13 英文 “Ins3.13.5”、中文“3.13.7”；3.43 一处英文 3.43.2、中文 3.42.2；3.2.5 一处英文 3.1.3、中文 3.2.1。核对后统一。</t>
         </is>
       </c>
     </row>
@@ -1657,17 +1657,17 @@
       </c>
       <c r="D40" s="2" t="inlineStr">
         <is>
-          <t>3.16、3.19、3.25 等脱保护后洗涤</t>
+          <t>版本说明 第 3 条</t>
         </is>
       </c>
       <c r="E40" s="2" t="inlineStr">
         <is>
-          <t>搅拌5±2 min（目标时间：10 min）</t>
+          <t>20±10 min (target: 10 min)</t>
         </is>
       </c>
       <c r="F40" s="2" t="inlineStr">
         <is>
-          <t>中文 ±2 min 配目标 10 min；英文同时写 “Stir for 5±2 min … After stirring for 5±2 min”，搅拌写了两遍。3.4 封端后洗涤也有英文 5 ± 2 min、中文 10 ± 2 min 的不一致。</t>
+          <t>版本说明写封端 DIPEA 参考加料时间目标 10 min，3.4.3 正文写 20 ± 10 min（目标 20 min）。</t>
         </is>
       </c>
     </row>
@@ -1687,17 +1687,17 @@
       </c>
       <c r="D41" s="3" t="inlineStr">
         <is>
-          <t>3.5 等哌啶溶液确认</t>
+          <t>3.17.8、3.26.8 活化</t>
         </is>
       </c>
       <c r="E41" s="3" t="inlineStr">
         <is>
-          <t>17.50%~22.50%</t>
+          <t>Maintain for NLT 15 min</t>
         </is>
       </c>
       <c r="F41" s="3" t="inlineStr">
         <is>
-          <t>浓度 NOR 17.50–22.50% 和温度 NOR 只写在中文，英文句没有数字。参数表和 PVP 也没有浓度 NOR。</t>
+          <t>英文 NLT 15 min（目标 20 min），中文 20 ± 5 min；参数表 NOR 15–25 min。中文优先，英文改为 20 ± 5 min。</t>
         </is>
       </c>
     </row>
@@ -1712,22 +1712,22 @@
       </c>
       <c r="C42" s="2" t="inlineStr">
         <is>
-          <t>低</t>
+          <t>中</t>
         </is>
       </c>
       <c r="D42" s="2" t="inlineStr">
         <is>
-          <t>3.17.1、3.20.1 等</t>
+          <t>3.0 预处理</t>
         </is>
       </c>
       <c r="E42" s="2" t="inlineStr">
         <is>
-          <t>95±5 rpm</t>
+          <t>搅拌5 min±5 min</t>
         </is>
       </c>
       <c r="F42" s="2" t="inlineStr">
         <is>
-          <t>其余活化罐搅拌都是 95 ± 10 rpm。</t>
+          <t>英文 5 ± 2 min，中文 5 ± 5 min。</t>
         </is>
       </c>
     </row>
@@ -1742,22 +1742,22 @@
       </c>
       <c r="C43" s="3" t="inlineStr">
         <is>
-          <t>低</t>
+          <t>中</t>
         </is>
       </c>
       <c r="D43" s="3" t="inlineStr">
         <is>
-          <t>原料信息表 3.37.1、3.37.5、3.38.1</t>
+          <t>3.16、3.19、3.25 等脱保护后洗涤</t>
         </is>
       </c>
       <c r="E43" s="3" t="inlineStr">
         <is>
-          <t>3.37.1</t>
+          <t>搅拌5±2 min（目标时间：10 min）</t>
         </is>
       </c>
       <c r="F43" s="3" t="inlineStr">
         <is>
-          <t>体积比（8、10、5）错填到“摩尔比”列。</t>
+          <t>中文 ±2 min 配目标 10 min；英文同时写 “Stir for 5±2 min … After stirring for 5±2 min”，搅拌写了两遍。3.4 封端后洗涤也有英文 5 ± 2 min、中文 10 ± 2 min 的不一致。</t>
         </is>
       </c>
     </row>
@@ -1772,22 +1772,22 @@
       </c>
       <c r="C44" s="2" t="inlineStr">
         <is>
-          <t>低</t>
+          <t>中</t>
         </is>
       </c>
       <c r="D44" s="2" t="inlineStr">
         <is>
-          <t>原料信息表 3.2.4 与 3.4.3</t>
+          <t>3.5 等哌啶溶液确认</t>
         </is>
       </c>
       <c r="E44" s="2" t="inlineStr">
         <is>
-          <t>129.24</t>
+          <t>17.50%~22.50%</t>
         </is>
       </c>
       <c r="F44" s="2" t="inlineStr">
         <is>
-          <t>DIPEA 分子量写 129.25 和 129.24 两个值。</t>
+          <t>浓度 NOR 17.50–22.50% 和温度 NOR 只写在中文，英文句没有数字。参数表和 PVP 也没有浓度 NOR。</t>
         </is>
       </c>
     </row>
@@ -1797,27 +1797,27 @@
       </c>
       <c r="B45" s="3" t="inlineStr">
         <is>
-          <t>中英翻译</t>
+          <t>内部数值/逻辑</t>
         </is>
       </c>
       <c r="C45" s="3" t="inlineStr">
         <is>
-          <t>高</t>
+          <t>低</t>
         </is>
       </c>
       <c r="D45" s="3" t="inlineStr">
         <is>
-          <t>全文（约 300 处）</t>
+          <t>3.17.1、3.20.1 等</t>
         </is>
       </c>
       <c r="E45" s="3" t="inlineStr">
         <is>
-          <t>用于工艺性能执行</t>
+          <t>95±5 rpm</t>
         </is>
       </c>
       <c r="F45" s="3" t="inlineStr">
         <is>
-          <t>“确认”被成批替换成“执行”，且 MOR 规定中文为准：如“工艺性能执行”（应为工艺性能确认，即 PPQ）、“执行物料在复检日期”、“操作人员须执行反应体系温度…”、“拉曼扫描执行”、“各类执行”、“设备执行和配方执行”、“执行合计净重在投料范围内”。全文把这类“执行”改回“确认”，“执行人及日期”除外。</t>
+          <t>其余活化罐搅拌都是 95 ± 10 rpm。</t>
         </is>
       </c>
     </row>
@@ -1827,27 +1827,27 @@
       </c>
       <c r="B46" s="2" t="inlineStr">
         <is>
-          <t>中英翻译</t>
+          <t>内部数值/逻辑</t>
         </is>
       </c>
       <c r="C46" s="2" t="inlineStr">
         <is>
-          <t>中</t>
+          <t>低</t>
         </is>
       </c>
       <c r="D46" s="2" t="inlineStr">
         <is>
-          <t>3.5.3、3.8.3、3.11.3</t>
+          <t>原料信息表 3.37.1、3.37.5、3.38.1</t>
         </is>
       </c>
       <c r="E46" s="2" t="inlineStr">
         <is>
-          <t>滤除至基本</t>
+          <t>3.37.1</t>
         </is>
       </c>
       <c r="F46" s="2" t="inlineStr">
         <is>
-          <t>中文“滤除至基本通过隔膜泵从合成釜中排出溶液”断句错乱；英文 “Filter until nearly no liquid outflow” 与后一句 Drain 重复。删去该半句。</t>
+          <t>体积比（8、10、5）错填到“摩尔比”列。</t>
         </is>
       </c>
     </row>
@@ -1857,27 +1857,27 @@
       </c>
       <c r="B47" s="3" t="inlineStr">
         <is>
-          <t>中英翻译</t>
+          <t>内部数值/逻辑</t>
         </is>
       </c>
       <c r="C47" s="3" t="inlineStr">
         <is>
-          <t>中</t>
+          <t>低</t>
         </is>
       </c>
       <c r="D47" s="3" t="inlineStr">
         <is>
-          <t>收料 Ins.4</t>
+          <t>原料信息表 3.2.4 与 3.4.3</t>
         </is>
       </c>
       <c r="E47" s="3" t="inlineStr">
         <is>
-          <t>Particulate Drain</t>
+          <t>129.24</t>
         </is>
       </c>
       <c r="F47" s="3" t="inlineStr">
         <is>
-          <t>颗粒物滤棉译成 Particulate Drain，应为 particulate filter（分装节已写对）。</t>
+          <t>DIPEA 分子量写 129.25 和 129.24 两个值。</t>
         </is>
       </c>
     </row>
@@ -1892,22 +1892,22 @@
       </c>
       <c r="C48" s="2" t="inlineStr">
         <is>
-          <t>中</t>
+          <t>高</t>
         </is>
       </c>
       <c r="D48" s="2" t="inlineStr">
         <is>
-          <t>收料 Ins.4 转移</t>
+          <t>全文（约 300 处）</t>
         </is>
       </c>
       <c r="E48" s="2" t="inlineStr">
         <is>
-          <t>use a cabinet when transferring</t>
+          <t>用于工艺性能执行</t>
         </is>
       </c>
       <c r="F48" s="2" t="inlineStr">
         <is>
-          <t>中文“保温箱”，英文 cabinet。2–8 °C 转移应为 insulated box / cool box。</t>
+          <t>“确认”被成批替换成“执行”，且 MOR 规定中文为准：如“工艺性能执行”（应为工艺性能确认，即 PPQ）、“执行物料在复检日期”、“操作人员须执行反应体系温度…”、“拉曼扫描执行”、“各类执行”、“设备执行和配方执行”、“执行合计净重在投料范围内”。全文把这类“执行”改回“确认”，“执行人及日期”除外。</t>
         </is>
       </c>
     </row>
@@ -1922,22 +1922,22 @@
       </c>
       <c r="C49" s="3" t="inlineStr">
         <is>
-          <t>低</t>
+          <t>中</t>
         </is>
       </c>
       <c r="D49" s="3" t="inlineStr">
         <is>
-          <t>英文缩写表</t>
+          <t>3.5.3、3.8.3、3.11.3</t>
         </is>
       </c>
       <c r="E49" s="3" t="inlineStr">
         <is>
-          <t>Qty</t>
+          <t>滤除至基本</t>
         </is>
       </c>
       <c r="F49" s="3" t="inlineStr">
         <is>
-          <t>Qty 的中文写“质量”，应为“数量”；缩写表缺 CPP、NOR、PAR、DMF、DIC、DIPEA、IPAc、MTBE、LDPE、HDPE、OEB、FIO 等正文实际用到的缩写，却列了没用到的 MP、BP。</t>
+          <t>中文“滤除至基本通过隔膜泵从合成釜中排出溶液”断句错乱；英文 “Filter until nearly no liquid outflow” 与后一句 Drain 重复。删去该半句。</t>
         </is>
       </c>
     </row>
@@ -1952,22 +1952,22 @@
       </c>
       <c r="C50" s="2" t="inlineStr">
         <is>
-          <t>低</t>
+          <t>中</t>
         </is>
       </c>
       <c r="D50" s="2" t="inlineStr">
         <is>
-          <t>3.18、3.21、3.24、3.27 取样</t>
+          <t>收料 Ins.4</t>
         </is>
       </c>
       <c r="E50" s="2" t="inlineStr">
         <is>
-          <t>Kaiser test record</t>
+          <t>Particulate Drain</t>
         </is>
       </c>
       <c r="F50" s="2" t="inlineStr">
         <is>
-          <t>其余偶联写 ninhydrin test record，这四处写 Kaiser test record，记录名统一。</t>
+          <t>颗粒物滤棉译成 Particulate Drain，应为 particulate filter（分装节已写对）。</t>
         </is>
       </c>
     </row>
@@ -1977,27 +1977,27 @@
       </c>
       <c r="B51" s="3" t="inlineStr">
         <is>
-          <t>笔误/格式</t>
+          <t>中英翻译</t>
         </is>
       </c>
       <c r="C51" s="3" t="inlineStr">
         <is>
-          <t>低</t>
+          <t>中</t>
         </is>
       </c>
       <c r="D51" s="3" t="inlineStr">
         <is>
-          <t>多处</t>
+          <t>收料 Ins.4 转移</t>
         </is>
       </c>
       <c r="E51" s="3" t="inlineStr">
         <is>
-          <t>Shirnk</t>
+          <t>use a cabinet when transferring</t>
         </is>
       </c>
       <c r="F51" s="3" t="inlineStr">
         <is>
-          <t>Shirnk（2 处）、soulution（3）、diaphragmgm（2）、Ddeprotection、Adust、activation tan、Pyriine（代码表）、hastelly、cleacing、Ckecked、Checeked、Checkmed（3）、Ttransfer、additon、Sloid、LDPEpowder、butunpack（2）、solutionand、drainingdiaphragm、“conten t”、“Solid-peptide peptide synthesizer”、“哈式合金”、3.46 中文标题前多一个“芴”、TJ4S-1213-Sy15-RT01。</t>
+          <t>中文“保温箱”，英文 cabinet。2–8 °C 转移应为 insulated box / cool box。</t>
         </is>
       </c>
     </row>
@@ -2007,27 +2007,27 @@
       </c>
       <c r="B52" s="2" t="inlineStr">
         <is>
-          <t>笔误/格式</t>
+          <t>中英翻译</t>
         </is>
       </c>
       <c r="C52" s="2" t="inlineStr">
         <is>
-          <t>低</t>
+          <t>中</t>
         </is>
       </c>
       <c r="D52" s="2" t="inlineStr">
         <is>
-          <t>分装各节</t>
+          <t>3.5.9、3.11.9、3.31.9</t>
         </is>
       </c>
       <c r="E52" s="2" t="inlineStr">
         <is>
-          <t>Page 32~62 of 624</t>
+          <t>3.5.9 Resin reswelling wash 1</t>
         </is>
       </c>
       <c r="F52" s="2" t="inlineStr">
         <is>
-          <t>文件共 674 页（30 处）。改页码或去掉总页数。</t>
+          <t>英文写 wash 1，中文写“洗涤2”（3.11.9 少一个“后”）。对照同结构的 3.8.9，英文是 wash 2、中文是洗涤2，前一步是加 DMF。MOR 以中文为准，这三处英文改为 wash 2；3.11.9 中文改为“溶胀后洗涤2”。</t>
         </is>
       </c>
     </row>
@@ -2037,7 +2037,7 @@
       </c>
       <c r="B53" s="3" t="inlineStr">
         <is>
-          <t>笔误/格式</t>
+          <t>中英翻译</t>
         </is>
       </c>
       <c r="C53" s="3" t="inlineStr">
@@ -2047,17 +2047,17 @@
       </c>
       <c r="D53" s="3" t="inlineStr">
         <is>
-          <t>3.40.3；3.45；目录 3.8、3.25</t>
+          <t>英文缩写表</t>
         </is>
       </c>
       <c r="E53" s="3" t="inlineStr">
         <is>
-          <t>Deprotection of Fmoc-L-Leu-OH activation</t>
+          <t>Qty</t>
         </is>
       </c>
       <c r="F53" s="3" t="inlineStr">
         <is>
-          <t>标题与内容不符：3.40.3 写“Leu 活化的脱保护”；3.45 只有再溶胀却叫 “(14) Deprotection”；目录 3.8、3.25 把脱保护标成下一个氨基酸名。3.43.5 编号用了两次。</t>
+          <t>Qty 的中文写“质量”，应为“数量”；缩写表缺 CPP、NOR、PAR、DMF、DIC、DIPEA、IPAc、MTBE、LDPE、HDPE、OEB、FIO 等正文实际用到的缩写，却列了没用到的 MP、BP。</t>
         </is>
       </c>
     </row>
@@ -2067,7 +2067,7 @@
       </c>
       <c r="B54" s="2" t="inlineStr">
         <is>
-          <t>笔误/格式</t>
+          <t>中英翻译</t>
         </is>
       </c>
       <c r="C54" s="2" t="inlineStr">
@@ -2077,17 +2077,17 @@
       </c>
       <c r="D54" s="2" t="inlineStr">
         <is>
-          <t>3.10.5</t>
+          <t>3.18、3.21、3.24、3.27 取样</t>
         </is>
       </c>
       <c r="E54" s="2" t="inlineStr">
         <is>
-          <t>(target: 4 h) (target：4 h)</t>
+          <t>Kaiser test record</t>
         </is>
       </c>
       <c r="F54" s="2" t="inlineStr">
         <is>
-          <t>目标重复写了两次。</t>
+          <t>其余偶联写 ninhydrin test record，这四处写 Kaiser test record，记录名统一。</t>
         </is>
       </c>
     </row>
@@ -2107,17 +2107,17 @@
       </c>
       <c r="D55" s="3" t="inlineStr">
         <is>
-          <t>3.6.5</t>
+          <t>多处</t>
         </is>
       </c>
       <c r="E55" s="3" t="inlineStr">
         <is>
-          <t>(target: 5 ℃.</t>
+          <t>Shirnk</t>
         </is>
       </c>
       <c r="F55" s="3" t="inlineStr">
         <is>
-          <t>括号没关。</t>
+          <t>Shirnk（2 处）、soulution（3）、diaphragmgm（2）、Ddeprotection、Adust、activation tan、Pyriine（代码表）、hastelly、cleacing、Ckecked、Checeked、Checkmed（3）、Ttransfer、additon、Sloid、LDPEpowder、butunpack（2）、solutionand、drainingdiaphragm、“conten t”、“Solid-peptide peptide synthesizer”、“哈式合金”、3.46 中文标题前多一个“芴”、TJ4S-1213-Sy15-RT01。</t>
         </is>
       </c>
     </row>
@@ -2137,17 +2137,17 @@
       </c>
       <c r="D56" s="2" t="inlineStr">
         <is>
-          <t>3.15.6</t>
+          <t>分装各节</t>
         </is>
       </c>
       <c r="E56" s="2" t="inlineStr">
         <is>
-          <t>Charge 364.03 kg DMF addition</t>
+          <t>Page 32~62 of 624</t>
         </is>
       </c>
       <c r="F56" s="2" t="inlineStr">
         <is>
-          <t>英文语法不通，且缺称量范围（中文有）。</t>
+          <t>文件共 674 页（30 处）。改页码或去掉总页数。</t>
         </is>
       </c>
     </row>
@@ -2167,22 +2167,142 @@
       </c>
       <c r="D57" s="3" t="inlineStr">
         <is>
+          <t>3.40.3；3.45；目录 3.8、3.25</t>
+        </is>
+      </c>
+      <c r="E57" s="3" t="inlineStr">
+        <is>
+          <t>Deprotection of Fmoc-L-Leu-OH activation</t>
+        </is>
+      </c>
+      <c r="F57" s="3" t="inlineStr">
+        <is>
+          <t>标题与内容不符：3.40.3 写“Leu 活化的脱保护”；3.45 只有再溶胀却叫 “(14) Deprotection”；目录 3.8、3.25 把脱保护标成下一个氨基酸名。3.43.5 编号用了两次。</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="2" t="n">
+        <v>57</v>
+      </c>
+      <c r="B58" s="2" t="inlineStr">
+        <is>
+          <t>笔误/格式</t>
+        </is>
+      </c>
+      <c r="C58" s="2" t="inlineStr">
+        <is>
+          <t>低</t>
+        </is>
+      </c>
+      <c r="D58" s="2" t="inlineStr">
+        <is>
+          <t>3.10.5</t>
+        </is>
+      </c>
+      <c r="E58" s="2" t="inlineStr">
+        <is>
+          <t>(target: 4 h) (target：4 h)</t>
+        </is>
+      </c>
+      <c r="F58" s="2" t="inlineStr">
+        <is>
+          <t>目标重复写了两次。</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="3" t="n">
+        <v>58</v>
+      </c>
+      <c r="B59" s="3" t="inlineStr">
+        <is>
+          <t>笔误/格式</t>
+        </is>
+      </c>
+      <c r="C59" s="3" t="inlineStr">
+        <is>
+          <t>低</t>
+        </is>
+      </c>
+      <c r="D59" s="3" t="inlineStr">
+        <is>
+          <t>3.6.5</t>
+        </is>
+      </c>
+      <c r="E59" s="3" t="inlineStr">
+        <is>
+          <t>(target: 5 ℃.</t>
+        </is>
+      </c>
+      <c r="F59" s="3" t="inlineStr">
+        <is>
+          <t>括号没关。</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="2" t="n">
+        <v>59</v>
+      </c>
+      <c r="B60" s="2" t="inlineStr">
+        <is>
+          <t>笔误/格式</t>
+        </is>
+      </c>
+      <c r="C60" s="2" t="inlineStr">
+        <is>
+          <t>低</t>
+        </is>
+      </c>
+      <c r="D60" s="2" t="inlineStr">
+        <is>
+          <t>3.15.6</t>
+        </is>
+      </c>
+      <c r="E60" s="2" t="inlineStr">
+        <is>
+          <t>Charge 364.03 kg DMF addition</t>
+        </is>
+      </c>
+      <c r="F60" s="2" t="inlineStr">
+        <is>
+          <t>英文语法不通，且缺称量范围（中文有）。</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="3" t="n">
+        <v>60</v>
+      </c>
+      <c r="B61" s="3" t="inlineStr">
+        <is>
+          <t>笔误/格式</t>
+        </is>
+      </c>
+      <c r="C61" s="3" t="inlineStr">
+        <is>
+          <t>低</t>
+        </is>
+      </c>
+      <c r="D61" s="3" t="inlineStr">
+        <is>
           <t>过程中间体信息</t>
         </is>
       </c>
-      <c r="E57" s="3" t="inlineStr">
+      <c r="E61" s="3" t="inlineStr">
         <is>
           <t>÷ 1000 kg/mol]</t>
         </is>
       </c>
-      <c r="F57" s="3" t="inlineStr">
+      <c r="F61" s="3" t="inlineStr">
         <is>
           <t>公式多一个 “]”。</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:F57"/>
+  <autoFilter ref="A1:F61"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
 </worksheet>

</xml_diff>